<commit_message>
Fix SQLAlchemy async errors, refactor Setup Wizard, and optimize Excel processing services
</commit_message>
<xml_diff>
--- a/_data_list/FF_MO.xlsx
+++ b/_data_list/FF_MO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Telegram_Project\OrangeFlow_Dev\_data_list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D142DB42-56E1-4E18-9C61-73D3655C0170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3F9E908-9413-4380-959F-1C0C9CDD54A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="85">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -1197,6 +1197,9 @@
       <c r="Q9" s="3">
         <v>2311580467330</v>
       </c>
+      <c r="AJ9" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -1217,6 +1220,9 @@
       <c r="K10" s="2"/>
       <c r="N10" s="2"/>
       <c r="Q10" s="3"/>
+      <c r="AJ10" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="K11" s="2"/>

</xml_diff>